<commit_message>
Update Swarnix subscription features spreadsheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Swarnix subscription features.xlsx
+++ b/public/Swarnix subscription features.xlsx
@@ -118,7 +118,7 @@
     <t>Free (For 15 days)</t>
   </si>
   <si>
-    <t>Rs. 3999 + GST</t>
+    <t>Rs. 4999 + GST</t>
   </si>
   <si>
     <t>Rs. 8999 + GST</t>
@@ -132,7 +132,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,6 +153,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -167,7 +173,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -188,6 +194,13 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -212,16 +225,16 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -535,7 +548,7 @@
     <col min="5" max="5" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -756,7 +769,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="3" t="s">
         <v>21</v>
       </c>
@@ -841,7 +854,7 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="3" t="s">
         <v>32</v>
       </c>

</xml_diff>

<commit_message>
Update Swarnix subscription features excel
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Swarnix subscription features.xlsx
+++ b/public/Swarnix subscription features.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="37">
   <si>
     <t>Per Month</t>
   </si>
@@ -22,6 +22,9 @@
     <t>Trial</t>
   </si>
   <si>
+    <t>Basic</t>
+  </si>
+  <si>
     <t>Starter</t>
   </si>
   <si>
@@ -31,7 +34,7 @@
     <t>Enterprise</t>
   </si>
   <si>
-    <t>Credits</t>
+    <t>Conversations</t>
   </si>
   <si>
     <t>Smart inventory App</t>
@@ -76,16 +79,13 @@
     <t>Customer Tiers (VVIP / VIP / Regular)</t>
   </si>
   <si>
-    <t>AI Models Try-On</t>
-  </si>
-  <si>
-    <t>Selfie Try-On for Customers</t>
-  </si>
-  <si>
-    <t>Design Your Jewellery</t>
-  </si>
-  <si>
-    <t>Website</t>
+    <t xml:space="preserve">AI Studio Suite
+(Studio Photo, Metal Swap, Jewellery Design,
+AI Models, Reels, Selfie Try-On for Customers)
+</t>
+  </si>
+  <si>
+    <t>Shared Website</t>
   </si>
   <si>
     <t>Team Members login</t>
@@ -97,13 +97,13 @@
     <t>Advanced</t>
   </si>
   <si>
-    <t>Basic</t>
-  </si>
-  <si>
     <t>Price</t>
   </si>
   <si>
     <t>Rs. 1999 + GST</t>
+  </si>
+  <si>
+    <t>Rs. 3999 + GST</t>
   </si>
   <si>
     <t>Rs. 6999 + GST</t>
@@ -210,7 +210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -218,12 +218,18 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -244,6 +250,9 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -547,14 +556,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="40.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="21.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="14.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="40.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="13" width="21.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="13" width="14.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="13" width="14.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -564,7 +574,7 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -573,328 +583,348 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="4">
+      <c r="A2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="5">
         <v>200</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="6">
+        <v>500</v>
+      </c>
+      <c r="D2" s="5">
         <v>1000</v>
       </c>
-      <c r="D2" s="4">
+      <c r="E2" s="5">
         <v>3000</v>
       </c>
-      <c r="E2" s="4">
+      <c r="F2" s="5">
         <v>10000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>7</v>
+      <c r="B3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>7</v>
+      <c r="A4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>7</v>
+      <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="4">
+      <c r="A6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="5">
         <v>100</v>
       </c>
-      <c r="C6" s="4">
-        <v>500</v>
-      </c>
-      <c r="D6" s="4">
+      <c r="C6" s="6">
+        <v>300</v>
+      </c>
+      <c r="D6" s="5">
         <v>1000</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="5">
+        <v>2000</v>
+      </c>
+      <c r="F6" s="5">
         <v>5000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>7</v>
+      <c r="A7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>14</v>
+      <c r="C8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>7</v>
+      <c r="A9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>7</v>
+      <c r="B10" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>7</v>
+      <c r="C11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="41.25">
+      <c r="A13" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="9">
         <v>20</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="6">
         <v>50</v>
       </c>
-      <c r="D13" s="4">
-        <v>200</v>
-      </c>
-      <c r="E13" s="4">
-        <v>500</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="4">
-        <v>10</v>
-      </c>
-      <c r="C14" s="4">
+      <c r="D13" s="9">
+        <v>150</v>
+      </c>
+      <c r="E13" s="9">
+        <v>400</v>
+      </c>
+      <c r="F13" s="9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="4">
-        <v>100</v>
-      </c>
-      <c r="E14" s="4">
-        <v>300</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="7">
-        <v>100</v>
-      </c>
-      <c r="E15" s="7">
-        <v>300</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="5" t="s">
+      <c r="F17" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+      <c r="A18" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
-      <c r="A20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="5" t="s">
+      <c r="D18" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="E18" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="F18" s="7" t="s">
         <v>36</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>